<commit_message>
biomass data and lovely code from Evan
</commit_message>
<xml_diff>
--- a/data/biomass/biomass_sla.xlsx
+++ b/data/biomass/biomass_sla.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\working\waccache\SN3PEPF00017C02\EXCELCNV\2eb75816-4298-4d6b-9669-3e96551616f1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://texastechuniversity-my.sharepoint.com/personal/monikell_ttu_edu/Documents/0_sorted_files/research/mk/exp_02/data/biomass/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{254185C5-46C9-489C-9FE3-1E477E2A10B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CCA7BB7-B2D1-4DC3-B3E6-E031514DA64D}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="8_{254185C5-46C9-489C-9FE3-1E477E2A10B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44C28281-65AB-431F-B6D2-3F3F8CF39FFB}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{4443427A-40C9-436B-A446-19B65A096950}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4443427A-40C9-436B-A446-19B65A096950}"/>
   </bookViews>
   <sheets>
     <sheet name="in" sheetId="1" r:id="rId1"/>
@@ -78,7 +78,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -616,9 +616,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -656,7 +656,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -762,7 +762,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -904,7 +904,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -913,12 +913,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{436253DA-0B4E-46B2-8791-75ACF98A9C76}">
   <dimension ref="A1:D390"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -932,7 +933,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -943,7 +944,7 @@
         <v>8.3799999999999999E-2</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -954,7 +955,7 @@
         <v>4.2000000000000003E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -965,7 +966,7 @@
         <v>3.44E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -976,7 +977,7 @@
         <v>8.4500000000000006E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -987,7 +988,7 @@
         <v>8.3500000000000005E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -998,7 +999,7 @@
         <v>6.5500000000000003E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1009,7 +1010,7 @@
         <v>6.2399999999999997E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -1020,7 +1021,7 @@
         <v>5.57E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -1031,7 +1032,7 @@
         <v>7.4999999999999997E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -1042,7 +1043,7 @@
         <v>2.8400000000000002E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -1053,7 +1054,7 @@
         <v>2.47E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -1064,7 +1065,7 @@
         <v>0.14000000000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -1075,7 +1076,7 @@
         <v>7.5300000000000006E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -1086,7 +1087,7 @@
         <v>5.4399999999999997E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -1097,7 +1098,7 @@
         <v>9.1300000000000006E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -1108,7 +1109,7 @@
         <v>9.9500000000000005E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -1119,7 +1120,7 @@
         <v>6.3799999999999996E-2</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -1130,7 +1131,7 @@
         <v>2.12E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -1141,7 +1142,7 @@
         <v>0.1095</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -1152,7 +1153,7 @@
         <v>6.8199999999999997E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -1163,7 +1164,7 @@
         <v>0.1152</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -1174,7 +1175,7 @@
         <v>6.1899999999999997E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -1185,7 +1186,7 @@
         <v>0.108</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>4</v>
       </c>
@@ -1196,7 +1197,7 @@
         <v>6.9699999999999998E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>4</v>
       </c>
@@ -1207,7 +1208,7 @@
         <v>0.1414</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>4</v>
       </c>
@@ -1218,7 +1219,7 @@
         <v>3.3599999999999998E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>4</v>
       </c>
@@ -1229,7 +1230,7 @@
         <v>5.2299999999999999E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>4</v>
       </c>
@@ -1240,7 +1241,7 @@
         <v>6.13E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>4</v>
       </c>
@@ -1251,7 +1252,7 @@
         <v>2.9700000000000001E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>4</v>
       </c>
@@ -1262,7 +1263,7 @@
         <v>5.67E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>4</v>
       </c>
@@ -1273,7 +1274,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>4</v>
       </c>
@@ -1284,7 +1285,7 @@
         <v>5.7200000000000001E-2</v>
       </c>
     </row>
-    <row r="34" spans="1:3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>4</v>
       </c>
@@ -1295,7 +1296,7 @@
         <v>2.4199999999999999E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>4</v>
       </c>
@@ -1306,7 +1307,7 @@
         <v>1.5900000000000001E-2</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>4</v>
       </c>
@@ -1317,7 +1318,7 @@
         <v>2.7099999999999999E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>4</v>
       </c>
@@ -1328,7 +1329,7 @@
         <v>5.1700000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>4</v>
       </c>
@@ -1339,7 +1340,7 @@
         <v>6.2100000000000002E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>4</v>
       </c>
@@ -1350,7 +1351,7 @@
         <v>3.8600000000000002E-2</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>4</v>
       </c>
@@ -1361,7 +1362,7 @@
         <v>1.2200000000000001E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>4</v>
       </c>
@@ -1372,7 +1373,7 @@
         <v>2.4899999999999999E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>4</v>
       </c>
@@ -1383,7 +1384,7 @@
         <v>5.4800000000000001E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>4</v>
       </c>
@@ -1394,7 +1395,7 @@
         <v>1.34E-2</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>4</v>
       </c>
@@ -1405,7 +1406,7 @@
         <v>6.2199999999999998E-2</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>4</v>
       </c>
@@ -1416,7 +1417,7 @@
         <v>3.3399999999999999E-2</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>4</v>
       </c>
@@ -1427,7 +1428,7 @@
         <v>6.0400000000000002E-2</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>4</v>
       </c>
@@ -1438,7 +1439,7 @@
         <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>4</v>
       </c>
@@ -1449,7 +1450,7 @@
         <v>4.1500000000000002E-2</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>4</v>
       </c>
@@ -1460,7 +1461,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -1471,7 +1472,7 @@
         <v>2.1600000000000001E-2</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>4</v>
       </c>
@@ -1482,7 +1483,7 @@
         <v>1.9E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>4</v>
       </c>
@@ -1493,7 +1494,7 @@
         <v>2.9700000000000001E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>4</v>
       </c>
@@ -1504,7 +1505,7 @@
         <v>3.4299999999999997E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>4</v>
       </c>
@@ -1515,7 +1516,7 @@
         <v>0.11210000000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>4</v>
       </c>
@@ -1526,7 +1527,7 @@
         <v>3.6600000000000001E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>4</v>
       </c>
@@ -1540,7 +1541,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>4</v>
       </c>
@@ -1551,7 +1552,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>4</v>
       </c>
@@ -1565,7 +1566,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>4</v>
       </c>
@@ -1576,7 +1577,7 @@
         <v>1.41E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>4</v>
       </c>
@@ -1587,7 +1588,7 @@
         <v>5.91E-2</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>4</v>
       </c>
@@ -1598,7 +1599,7 @@
         <v>2.2100000000000002E-2</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>4</v>
       </c>
@@ -1609,7 +1610,7 @@
         <v>6.6000000000000003E-2</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>4</v>
       </c>
@@ -1620,7 +1621,7 @@
         <v>1.84E-2</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>4</v>
       </c>
@@ -1631,7 +1632,7 @@
         <v>1.0699999999999999E-2</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>4</v>
       </c>
@@ -1642,7 +1643,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>4</v>
       </c>
@@ -1653,7 +1654,7 @@
         <v>8.7800000000000003E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>4</v>
       </c>
@@ -1664,7 +1665,7 @@
         <v>2.5100000000000001E-2</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>4</v>
       </c>
@@ -1675,7 +1676,7 @@
         <v>5.2200000000000003E-2</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>4</v>
       </c>
@@ -1686,7 +1687,7 @@
         <v>7.9299999999999995E-2</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>4</v>
       </c>
@@ -1697,7 +1698,7 @@
         <v>0.1164</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>4</v>
       </c>
@@ -1708,7 +1709,7 @@
         <v>3.09E-2</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>4</v>
       </c>
@@ -1719,7 +1720,7 @@
         <v>6.5600000000000006E-2</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>4</v>
       </c>
@@ -1730,7 +1731,7 @@
         <v>6.2600000000000003E-2</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>4</v>
       </c>
@@ -1741,7 +1742,7 @@
         <v>0.1406</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>4</v>
       </c>
@@ -1752,7 +1753,7 @@
         <v>2.53E-2</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>4</v>
       </c>
@@ -1763,7 +1764,7 @@
         <v>3.7100000000000001E-2</v>
       </c>
     </row>
-    <row r="77" spans="1:3">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>4</v>
       </c>
@@ -1774,7 +1775,7 @@
         <v>5.7700000000000001E-2</v>
       </c>
     </row>
-    <row r="78" spans="1:3">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>4</v>
       </c>
@@ -1785,7 +1786,7 @@
         <v>8.0100000000000005E-2</v>
       </c>
     </row>
-    <row r="79" spans="1:3">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>4</v>
       </c>
@@ -1796,7 +1797,7 @@
         <v>4.1599999999999998E-2</v>
       </c>
     </row>
-    <row r="80" spans="1:3">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>4</v>
       </c>
@@ -1807,7 +1808,7 @@
         <v>6.9800000000000001E-2</v>
       </c>
     </row>
-    <row r="81" spans="1:3">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>4</v>
       </c>
@@ -1818,7 +1819,7 @@
         <v>7.4899999999999994E-2</v>
       </c>
     </row>
-    <row r="82" spans="1:3">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>4</v>
       </c>
@@ -1829,7 +1830,7 @@
         <v>6.8400000000000002E-2</v>
       </c>
     </row>
-    <row r="83" spans="1:3">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>4</v>
       </c>
@@ -1840,7 +1841,7 @@
         <v>2.2200000000000001E-2</v>
       </c>
     </row>
-    <row r="84" spans="1:3">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>4</v>
       </c>
@@ -1851,7 +1852,7 @@
         <v>4.4900000000000002E-2</v>
       </c>
     </row>
-    <row r="85" spans="1:3">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>4</v>
       </c>
@@ -1862,7 +1863,7 @@
         <v>0.1152</v>
       </c>
     </row>
-    <row r="86" spans="1:3">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>4</v>
       </c>
@@ -1873,7 +1874,7 @@
         <v>7.9899999999999999E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:3">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>4</v>
       </c>
@@ -1884,7 +1885,7 @@
         <v>5.9700000000000003E-2</v>
       </c>
     </row>
-    <row r="88" spans="1:3">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>4</v>
       </c>
@@ -1895,7 +1896,7 @@
         <v>4.6300000000000001E-2</v>
       </c>
     </row>
-    <row r="89" spans="1:3">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>4</v>
       </c>
@@ -1906,7 +1907,7 @@
         <v>8.9899999999999994E-2</v>
       </c>
     </row>
-    <row r="90" spans="1:3">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>4</v>
       </c>
@@ -1917,7 +1918,7 @@
         <v>0.13059999999999999</v>
       </c>
     </row>
-    <row r="91" spans="1:3">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>4</v>
       </c>
@@ -1928,7 +1929,7 @@
         <v>2.8000000000000001E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:3">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>4</v>
       </c>
@@ -1939,7 +1940,7 @@
         <v>3.78E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:3">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>4</v>
       </c>
@@ -1950,7 +1951,7 @@
         <v>6.7400000000000002E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:3">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>4</v>
       </c>
@@ -1961,7 +1962,7 @@
         <v>0.1148</v>
       </c>
     </row>
-    <row r="95" spans="1:3">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>4</v>
       </c>
@@ -1972,7 +1973,7 @@
         <v>4.3499999999999997E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:3">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>4</v>
       </c>
@@ -1983,7 +1984,7 @@
         <v>5.8999999999999997E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:3">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>4</v>
       </c>
@@ -1994,7 +1995,7 @@
         <v>6.8500000000000005E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:3">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>4</v>
       </c>
@@ -2005,7 +2006,7 @@
         <v>2.2499999999999999E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:3">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>4</v>
       </c>
@@ -2016,7 +2017,7 @@
         <v>2.6100000000000002E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:3">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>4</v>
       </c>
@@ -2027,7 +2028,7 @@
         <v>4.8899999999999999E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:3">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>4</v>
       </c>
@@ -2038,7 +2039,7 @@
         <v>2.9000000000000001E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:3">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>4</v>
       </c>
@@ -2049,7 +2050,7 @@
         <v>0.1038</v>
       </c>
     </row>
-    <row r="103" spans="1:3">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>4</v>
       </c>
@@ -2060,7 +2061,7 @@
         <v>3.5700000000000003E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:3">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>4</v>
       </c>
@@ -2071,7 +2072,7 @@
         <v>1.6799999999999999E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:3">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>4</v>
       </c>
@@ -2082,7 +2083,7 @@
         <v>3.4299999999999997E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:3">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>4</v>
       </c>
@@ -2093,7 +2094,7 @@
         <v>2.2200000000000001E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:3">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>4</v>
       </c>
@@ -2104,7 +2105,7 @@
         <v>2.0500000000000001E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:3">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>4</v>
       </c>
@@ -2115,7 +2116,7 @@
         <v>6.4500000000000002E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:3">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>4</v>
       </c>
@@ -2126,7 +2127,7 @@
         <v>7.9100000000000004E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:3">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>4</v>
       </c>
@@ -2137,7 +2138,7 @@
         <v>8.9700000000000002E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:3">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>4</v>
       </c>
@@ -2148,7 +2149,7 @@
         <v>3.8600000000000002E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:3">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>4</v>
       </c>
@@ -2159,7 +2160,7 @@
         <v>6.1600000000000002E-2</v>
       </c>
     </row>
-    <row r="113" spans="1:3">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>4</v>
       </c>
@@ -2170,7 +2171,7 @@
         <v>3.44E-2</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>4</v>
       </c>
@@ -2181,7 +2182,7 @@
         <v>7.6399999999999996E-2</v>
       </c>
     </row>
-    <row r="115" spans="1:3">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>4</v>
       </c>
@@ -2192,7 +2193,7 @@
         <v>2.29E-2</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>4</v>
       </c>
@@ -2203,7 +2204,7 @@
         <v>6.8500000000000005E-2</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>4</v>
       </c>
@@ -2214,7 +2215,7 @@
         <v>3.2800000000000003E-2</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>4</v>
       </c>
@@ -2225,7 +2226,7 @@
         <v>5.4199999999999998E-2</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>4</v>
       </c>
@@ -2236,7 +2237,7 @@
         <v>4.3200000000000002E-2</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>4</v>
       </c>
@@ -2247,7 +2248,7 @@
         <v>4.3700000000000003E-2</v>
       </c>
     </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>4</v>
       </c>
@@ -2258,7 +2259,7 @@
         <v>1.66E-2</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>4</v>
       </c>
@@ -2269,7 +2270,7 @@
         <v>3.4799999999999998E-2</v>
       </c>
     </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>4</v>
       </c>
@@ -2280,7 +2281,7 @@
         <v>2.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="124" spans="1:3">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>4</v>
       </c>
@@ -2291,7 +2292,7 @@
         <v>6.59E-2</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>4</v>
       </c>
@@ -2302,7 +2303,7 @@
         <v>5.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>4</v>
       </c>
@@ -2313,7 +2314,7 @@
         <v>6.6699999999999995E-2</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>4</v>
       </c>
@@ -2324,7 +2325,7 @@
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
-    <row r="128" spans="1:3">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>4</v>
       </c>
@@ -2335,7 +2336,7 @@
         <v>2.5600000000000001E-2</v>
       </c>
     </row>
-    <row r="129" spans="1:3">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>4</v>
       </c>
@@ -2346,7 +2347,7 @@
         <v>4.0399999999999998E-2</v>
       </c>
     </row>
-    <row r="130" spans="1:3">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>4</v>
       </c>
@@ -2357,7 +2358,7 @@
         <v>0.1018</v>
       </c>
     </row>
-    <row r="131" spans="1:3">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>4</v>
       </c>
@@ -2368,7 +2369,7 @@
         <v>2.5000000000000001E-2</v>
       </c>
     </row>
-    <row r="132" spans="1:3">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>4</v>
       </c>
@@ -2379,7 +2380,7 @@
         <v>3.5499999999999997E-2</v>
       </c>
     </row>
-    <row r="133" spans="1:3">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>4</v>
       </c>
@@ -2390,7 +2391,7 @@
         <v>4.8099999999999997E-2</v>
       </c>
     </row>
-    <row r="134" spans="1:3">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>4</v>
       </c>
@@ -2401,7 +2402,7 @@
         <v>9.6600000000000005E-2</v>
       </c>
     </row>
-    <row r="135" spans="1:3">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>4</v>
       </c>
@@ -2412,7 +2413,7 @@
         <v>4.6199999999999998E-2</v>
       </c>
     </row>
-    <row r="136" spans="1:3">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>4</v>
       </c>
@@ -2423,7 +2424,7 @@
         <v>8.7300000000000003E-2</v>
       </c>
     </row>
-    <row r="137" spans="1:3">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>4</v>
       </c>
@@ -2434,7 +2435,7 @@
         <v>7.7799999999999994E-2</v>
       </c>
     </row>
-    <row r="138" spans="1:3">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>4</v>
       </c>
@@ -2445,7 +2446,7 @@
         <v>0.1203</v>
       </c>
     </row>
-    <row r="139" spans="1:3">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>4</v>
       </c>
@@ -2456,7 +2457,7 @@
         <v>3.4799999999999998E-2</v>
       </c>
     </row>
-    <row r="140" spans="1:3">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>4</v>
       </c>
@@ -2467,7 +2468,7 @@
         <v>0.1023</v>
       </c>
     </row>
-    <row r="141" spans="1:3">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>4</v>
       </c>
@@ -2478,7 +2479,7 @@
         <v>6.2899999999999998E-2</v>
       </c>
     </row>
-    <row r="142" spans="1:3">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>4</v>
       </c>
@@ -2489,7 +2490,7 @@
         <v>8.7800000000000003E-2</v>
       </c>
     </row>
-    <row r="143" spans="1:3">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>4</v>
       </c>
@@ -2500,7 +2501,7 @@
         <v>6.6000000000000003E-2</v>
       </c>
     </row>
-    <row r="144" spans="1:3">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>4</v>
       </c>
@@ -2511,7 +2512,7 @@
         <v>9.0899999999999995E-2</v>
       </c>
     </row>
-    <row r="145" spans="1:4">
+    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>4</v>
       </c>
@@ -2522,7 +2523,7 @@
         <v>4.8599999999999997E-2</v>
       </c>
     </row>
-    <row r="146" spans="1:4">
+    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>4</v>
       </c>
@@ -2533,7 +2534,7 @@
         <v>7.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="147" spans="1:4">
+    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>4</v>
       </c>
@@ -2544,7 +2545,7 @@
         <v>2.4500000000000001E-2</v>
       </c>
     </row>
-    <row r="148" spans="1:4">
+    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>4</v>
       </c>
@@ -2555,7 +2556,7 @@
         <v>5.28E-2</v>
       </c>
     </row>
-    <row r="149" spans="1:4">
+    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>4</v>
       </c>
@@ -2566,7 +2567,7 @@
         <v>7.6899999999999996E-2</v>
       </c>
     </row>
-    <row r="150" spans="1:4">
+    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>4</v>
       </c>
@@ -2577,7 +2578,7 @@
         <v>9.0800000000000006E-2</v>
       </c>
     </row>
-    <row r="151" spans="1:4">
+    <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>4</v>
       </c>
@@ -2588,7 +2589,7 @@
         <v>5.67E-2</v>
       </c>
     </row>
-    <row r="152" spans="1:4">
+    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>4</v>
       </c>
@@ -2599,7 +2600,7 @@
         <v>0.10150000000000001</v>
       </c>
     </row>
-    <row r="153" spans="1:4">
+    <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>4</v>
       </c>
@@ -2613,7 +2614,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="154" spans="1:4">
+    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>4</v>
       </c>
@@ -2624,7 +2625,7 @@
         <v>0.16209999999999999</v>
       </c>
     </row>
-    <row r="155" spans="1:4">
+    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>4</v>
       </c>
@@ -2635,7 +2636,7 @@
         <v>2.7300000000000001E-2</v>
       </c>
     </row>
-    <row r="156" spans="1:4">
+    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>4</v>
       </c>
@@ -2646,7 +2647,7 @@
         <v>4.4200000000000003E-2</v>
       </c>
     </row>
-    <row r="157" spans="1:4">
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>4</v>
       </c>
@@ -2657,7 +2658,7 @@
         <v>6.7400000000000002E-2</v>
       </c>
     </row>
-    <row r="158" spans="1:4">
+    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>4</v>
       </c>
@@ -2668,7 +2669,7 @@
         <v>0.1101</v>
       </c>
     </row>
-    <row r="159" spans="1:4">
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>4</v>
       </c>
@@ -2679,7 +2680,7 @@
         <v>5.0900000000000001E-2</v>
       </c>
     </row>
-    <row r="160" spans="1:4">
+    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>4</v>
       </c>
@@ -2690,7 +2691,7 @@
         <v>6.25E-2</v>
       </c>
     </row>
-    <row r="161" spans="1:3">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>4</v>
       </c>
@@ -2701,7 +2702,7 @@
         <v>7.4899999999999994E-2</v>
       </c>
     </row>
-    <row r="162" spans="1:3">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>4</v>
       </c>
@@ -2712,7 +2713,7 @@
         <v>3.49E-2</v>
       </c>
     </row>
-    <row r="163" spans="1:3">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>4</v>
       </c>
@@ -2723,7 +2724,7 @@
         <v>2.1299999999999999E-2</v>
       </c>
     </row>
-    <row r="164" spans="1:3">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>4</v>
       </c>
@@ -2734,7 +2735,7 @@
         <v>4.1200000000000001E-2</v>
       </c>
     </row>
-    <row r="165" spans="1:3">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>4</v>
       </c>
@@ -2745,7 +2746,7 @@
         <v>2.75E-2</v>
       </c>
     </row>
-    <row r="166" spans="1:3">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>4</v>
       </c>
@@ -2756,7 +2757,7 @@
         <v>8.3900000000000002E-2</v>
       </c>
     </row>
-    <row r="167" spans="1:3">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>4</v>
       </c>
@@ -2767,7 +2768,7 @@
         <v>2.5700000000000001E-2</v>
       </c>
     </row>
-    <row r="168" spans="1:3">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>4</v>
       </c>
@@ -2778,7 +2779,7 @@
         <v>2.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="169" spans="1:3">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>4</v>
       </c>
@@ -2789,7 +2790,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="170" spans="1:3">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>4</v>
       </c>
@@ -2800,7 +2801,7 @@
         <v>9.6500000000000002E-2</v>
       </c>
     </row>
-    <row r="171" spans="1:3">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>4</v>
       </c>
@@ -2811,7 +2812,7 @@
         <v>1.7000000000000001E-2</v>
       </c>
     </row>
-    <row r="172" spans="1:3">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>4</v>
       </c>
@@ -2822,7 +2823,7 @@
         <v>6.4500000000000002E-2</v>
       </c>
     </row>
-    <row r="173" spans="1:3">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>4</v>
       </c>
@@ -2833,7 +2834,7 @@
         <v>2.52E-2</v>
       </c>
     </row>
-    <row r="174" spans="1:3">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>4</v>
       </c>
@@ -2844,7 +2845,7 @@
         <v>6.25E-2</v>
       </c>
     </row>
-    <row r="175" spans="1:3">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>4</v>
       </c>
@@ -2855,7 +2856,7 @@
         <v>3.1099999999999999E-2</v>
       </c>
     </row>
-    <row r="176" spans="1:3">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>4</v>
       </c>
@@ -2866,7 +2867,7 @@
         <v>1.2500000000000001E-2</v>
       </c>
     </row>
-    <row r="177" spans="1:3">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>4</v>
       </c>
@@ -2877,7 +2878,7 @@
         <v>2.6100000000000002E-2</v>
       </c>
     </row>
-    <row r="178" spans="1:3">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>4</v>
       </c>
@@ -2888,7 +2889,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="179" spans="1:3">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>4</v>
       </c>
@@ -2899,7 +2900,7 @@
         <v>1.9300000000000001E-2</v>
       </c>
     </row>
-    <row r="180" spans="1:3">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>4</v>
       </c>
@@ -2910,7 +2911,7 @@
         <v>6.4299999999999996E-2</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>4</v>
       </c>
@@ -2921,7 +2922,7 @@
         <v>4.3900000000000002E-2</v>
       </c>
     </row>
-    <row r="182" spans="1:3">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>4</v>
       </c>
@@ -2932,7 +2933,7 @@
         <v>6.5299999999999997E-2</v>
       </c>
     </row>
-    <row r="183" spans="1:3">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>4</v>
       </c>
@@ -2943,7 +2944,7 @@
         <v>3.6900000000000002E-2</v>
       </c>
     </row>
-    <row r="184" spans="1:3">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>4</v>
       </c>
@@ -2954,7 +2955,7 @@
         <v>4.0099999999999997E-2</v>
       </c>
     </row>
-    <row r="185" spans="1:3">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>4</v>
       </c>
@@ -2965,7 +2966,7 @@
         <v>3.2399999999999998E-2</v>
       </c>
     </row>
-    <row r="186" spans="1:3">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>4</v>
       </c>
@@ -2976,7 +2977,7 @@
         <v>1.9199999999999998E-2</v>
       </c>
     </row>
-    <row r="187" spans="1:3">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>4</v>
       </c>
@@ -2987,7 +2988,7 @@
         <v>1.37E-2</v>
       </c>
     </row>
-    <row r="188" spans="1:3">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>4</v>
       </c>
@@ -2998,7 +2999,7 @@
         <v>4.9799999999999997E-2</v>
       </c>
     </row>
-    <row r="189" spans="1:3">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>4</v>
       </c>
@@ -3009,7 +3010,7 @@
         <v>4.1799999999999997E-2</v>
       </c>
     </row>
-    <row r="190" spans="1:3">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>4</v>
       </c>
@@ -3020,7 +3021,7 @@
         <v>8.1799999999999998E-2</v>
       </c>
     </row>
-    <row r="191" spans="1:3">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>4</v>
       </c>
@@ -3031,7 +3032,7 @@
         <v>3.09E-2</v>
       </c>
     </row>
-    <row r="192" spans="1:3">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>4</v>
       </c>
@@ -3042,7 +3043,7 @@
         <v>2.63E-2</v>
       </c>
     </row>
-    <row r="193" spans="1:3">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>4</v>
       </c>
@@ -3053,7 +3054,7 @@
         <v>2.7199999999999998E-2</v>
       </c>
     </row>
-    <row r="194" spans="1:3">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>4</v>
       </c>
@@ -3064,7 +3065,7 @@
         <v>0.1065</v>
       </c>
     </row>
-    <row r="195" spans="1:3">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>4</v>
       </c>
@@ -3075,7 +3076,7 @@
         <v>3.7400000000000003E-2</v>
       </c>
     </row>
-    <row r="196" spans="1:3">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>4</v>
       </c>
@@ -3086,7 +3087,7 @@
         <v>3.73E-2</v>
       </c>
     </row>
-    <row r="197" spans="1:3">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>4</v>
       </c>
@@ -3097,7 +3098,7 @@
         <v>5.4199999999999998E-2</v>
       </c>
     </row>
-    <row r="198" spans="1:3">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>4</v>
       </c>
@@ -3108,7 +3109,7 @@
         <v>7.22E-2</v>
       </c>
     </row>
-    <row r="199" spans="1:3">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>4</v>
       </c>
@@ -3119,7 +3120,7 @@
         <v>3.85E-2</v>
       </c>
     </row>
-    <row r="200" spans="1:3">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>4</v>
       </c>
@@ -3130,7 +3131,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="201" spans="1:3">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>4</v>
       </c>
@@ -3141,7 +3142,7 @@
         <v>9.0899999999999995E-2</v>
       </c>
     </row>
-    <row r="202" spans="1:3">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>4</v>
       </c>
@@ -3152,7 +3153,7 @@
         <v>5.7799999999999997E-2</v>
       </c>
     </row>
-    <row r="203" spans="1:3">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>4</v>
       </c>
@@ -3163,7 +3164,7 @@
         <v>3.95E-2</v>
       </c>
     </row>
-    <row r="204" spans="1:3">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>4</v>
       </c>
@@ -3174,7 +3175,7 @@
         <v>8.5999999999999993E-2</v>
       </c>
     </row>
-    <row r="205" spans="1:3">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>4</v>
       </c>
@@ -3185,7 +3186,7 @@
         <v>3.9E-2</v>
       </c>
     </row>
-    <row r="206" spans="1:3">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>4</v>
       </c>
@@ -3196,7 +3197,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="207" spans="1:3">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>4</v>
       </c>
@@ -3207,7 +3208,7 @@
         <v>4.5699999999999998E-2</v>
       </c>
     </row>
-    <row r="208" spans="1:3">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>4</v>
       </c>
@@ -3218,7 +3219,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="209" spans="1:3">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>4</v>
       </c>
@@ -3229,7 +3230,7 @@
         <v>3.56E-2</v>
       </c>
     </row>
-    <row r="210" spans="1:3">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>4</v>
       </c>
@@ -3240,7 +3241,7 @@
         <v>0.11700000000000001</v>
       </c>
     </row>
-    <row r="211" spans="1:3">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>4</v>
       </c>
@@ -3251,7 +3252,7 @@
         <v>3.0200000000000001E-2</v>
       </c>
     </row>
-    <row r="212" spans="1:3">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>4</v>
       </c>
@@ -3262,7 +3263,7 @@
         <v>7.8899999999999998E-2</v>
       </c>
     </row>
-    <row r="213" spans="1:3">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>4</v>
       </c>
@@ -3273,7 +3274,7 @@
         <v>5.0099999999999999E-2</v>
       </c>
     </row>
-    <row r="214" spans="1:3">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>4</v>
       </c>
@@ -3284,7 +3285,7 @@
         <v>7.9299999999999995E-2</v>
       </c>
     </row>
-    <row r="215" spans="1:3">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>4</v>
       </c>
@@ -3295,7 +3296,7 @@
         <v>5.3100000000000001E-2</v>
       </c>
     </row>
-    <row r="216" spans="1:3">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>4</v>
       </c>
@@ -3306,7 +3307,7 @@
         <v>6.8699999999999997E-2</v>
       </c>
     </row>
-    <row r="217" spans="1:3">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>4</v>
       </c>
@@ -3317,7 +3318,7 @@
         <v>7.0400000000000004E-2</v>
       </c>
     </row>
-    <row r="218" spans="1:3">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>4</v>
       </c>
@@ -3328,7 +3329,7 @@
         <v>8.4400000000000003E-2</v>
       </c>
     </row>
-    <row r="219" spans="1:3">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>4</v>
       </c>
@@ -3339,7 +3340,7 @@
         <v>4.4299999999999999E-2</v>
       </c>
     </row>
-    <row r="220" spans="1:3">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>4</v>
       </c>
@@ -3350,7 +3351,7 @@
         <v>5.3800000000000001E-2</v>
       </c>
     </row>
-    <row r="221" spans="1:3">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>4</v>
       </c>
@@ -3361,7 +3362,7 @@
         <v>9.7799999999999998E-2</v>
       </c>
     </row>
-    <row r="222" spans="1:3">
+    <row r="222" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>4</v>
       </c>
@@ -3372,7 +3373,7 @@
         <v>7.2700000000000001E-2</v>
       </c>
     </row>
-    <row r="223" spans="1:3">
+    <row r="223" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>4</v>
       </c>
@@ -3383,7 +3384,7 @@
         <v>4.82E-2</v>
       </c>
     </row>
-    <row r="224" spans="1:3">
+    <row r="224" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>4</v>
       </c>
@@ -3394,7 +3395,7 @@
         <v>7.3999999999999996E-2</v>
       </c>
     </row>
-    <row r="225" spans="1:3">
+    <row r="225" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>4</v>
       </c>
@@ -3405,7 +3406,7 @@
         <v>6.5299999999999997E-2</v>
       </c>
     </row>
-    <row r="226" spans="1:3">
+    <row r="226" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>4</v>
       </c>
@@ -3416,7 +3417,7 @@
         <v>5.3100000000000001E-2</v>
       </c>
     </row>
-    <row r="227" spans="1:3">
+    <row r="227" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>4</v>
       </c>
@@ -3427,7 +3428,7 @@
         <v>1.9400000000000001E-2</v>
       </c>
     </row>
-    <row r="228" spans="1:3">
+    <row r="228" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>4</v>
       </c>
@@ -3438,7 +3439,7 @@
         <v>5.8099999999999999E-2</v>
       </c>
     </row>
-    <row r="229" spans="1:3">
+    <row r="229" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>4</v>
       </c>
@@ -3449,7 +3450,7 @@
         <v>2.1000000000000001E-2</v>
       </c>
     </row>
-    <row r="230" spans="1:3">
+    <row r="230" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>4</v>
       </c>
@@ -3460,7 +3461,7 @@
         <v>4.0899999999999999E-2</v>
       </c>
     </row>
-    <row r="231" spans="1:3">
+    <row r="231" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>4</v>
       </c>
@@ -3471,7 +3472,7 @@
         <v>3.78E-2</v>
       </c>
     </row>
-    <row r="232" spans="1:3">
+    <row r="232" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>4</v>
       </c>
@@ -3482,7 +3483,7 @@
         <v>3.5499999999999997E-2</v>
       </c>
     </row>
-    <row r="233" spans="1:3">
+    <row r="233" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>4</v>
       </c>
@@ -3493,7 +3494,7 @@
         <v>2.46E-2</v>
       </c>
     </row>
-    <row r="234" spans="1:3">
+    <row r="234" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>4</v>
       </c>
@@ -3504,7 +3505,7 @@
         <v>6.4500000000000002E-2</v>
       </c>
     </row>
-    <row r="235" spans="1:3">
+    <row r="235" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>4</v>
       </c>
@@ -3515,7 +3516,7 @@
         <v>1.6799999999999999E-2</v>
       </c>
     </row>
-    <row r="236" spans="1:3">
+    <row r="236" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>4</v>
       </c>
@@ -3526,7 +3527,7 @@
         <v>5.7500000000000002E-2</v>
       </c>
     </row>
-    <row r="237" spans="1:3">
+    <row r="237" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>4</v>
       </c>
@@ -3537,7 +3538,7 @@
         <v>4.0500000000000001E-2</v>
       </c>
     </row>
-    <row r="238" spans="1:3">
+    <row r="238" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>4</v>
       </c>
@@ -3548,7 +3549,7 @@
         <v>2.46E-2</v>
       </c>
     </row>
-    <row r="239" spans="1:3">
+    <row r="239" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>4</v>
       </c>
@@ -3559,7 +3560,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="240" spans="1:3">
+    <row r="240" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>4</v>
       </c>
@@ -3570,7 +3571,7 @@
         <v>2.5700000000000001E-2</v>
       </c>
     </row>
-    <row r="241" spans="1:3">
+    <row r="241" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>4</v>
       </c>
@@ -3581,7 +3582,7 @@
         <v>2.4199999999999999E-2</v>
       </c>
     </row>
-    <row r="242" spans="1:3">
+    <row r="242" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>4</v>
       </c>
@@ -3592,7 +3593,7 @@
         <v>1.2800000000000001E-2</v>
       </c>
     </row>
-    <row r="243" spans="1:3">
+    <row r="243" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>4</v>
       </c>
@@ -3603,7 +3604,7 @@
         <v>4.7000000000000002E-3</v>
       </c>
     </row>
-    <row r="244" spans="1:3">
+    <row r="244" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>4</v>
       </c>
@@ -3614,7 +3615,7 @@
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
-    <row r="245" spans="1:3">
+    <row r="245" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>4</v>
       </c>
@@ -3625,7 +3626,7 @@
         <v>1.5900000000000001E-2</v>
       </c>
     </row>
-    <row r="246" spans="1:3">
+    <row r="246" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>4</v>
       </c>
@@ -3636,7 +3637,7 @@
         <v>6.88E-2</v>
       </c>
     </row>
-    <row r="247" spans="1:3">
+    <row r="247" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>4</v>
       </c>
@@ -3647,7 +3648,7 @@
         <v>3.5299999999999998E-2</v>
       </c>
     </row>
-    <row r="248" spans="1:3">
+    <row r="248" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>4</v>
       </c>
@@ -3658,7 +3659,7 @@
         <v>4.6199999999999998E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:3">
+    <row r="249" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>4</v>
       </c>
@@ -3669,7 +3670,7 @@
         <v>2.58E-2</v>
       </c>
     </row>
-    <row r="250" spans="1:3">
+    <row r="250" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>4</v>
       </c>
@@ -3680,7 +3681,7 @@
         <v>2.4299999999999999E-2</v>
       </c>
     </row>
-    <row r="251" spans="1:3">
+    <row r="251" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>4</v>
       </c>
@@ -3691,7 +3692,7 @@
         <v>1.89E-2</v>
       </c>
     </row>
-    <row r="252" spans="1:3">
+    <row r="252" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>4</v>
       </c>
@@ -3702,7 +3703,7 @@
         <v>5.11E-2</v>
       </c>
     </row>
-    <row r="253" spans="1:3">
+    <row r="253" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>4</v>
       </c>
@@ -3713,7 +3714,7 @@
         <v>1.72E-2</v>
       </c>
     </row>
-    <row r="254" spans="1:3">
+    <row r="254" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>4</v>
       </c>
@@ -3724,7 +3725,7 @@
         <v>6.8199999999999997E-2</v>
       </c>
     </row>
-    <row r="255" spans="1:3">
+    <row r="255" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>4</v>
       </c>
@@ -3735,7 +3736,7 @@
         <v>2.07E-2</v>
       </c>
     </row>
-    <row r="256" spans="1:3">
+    <row r="256" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>4</v>
       </c>
@@ -3746,7 +3747,7 @@
         <v>5.3100000000000001E-2</v>
       </c>
     </row>
-    <row r="257" spans="1:3">
+    <row r="257" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>4</v>
       </c>
@@ -3757,7 +3758,7 @@
         <v>5.7200000000000001E-2</v>
       </c>
     </row>
-    <row r="258" spans="1:3">
+    <row r="258" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>4</v>
       </c>
@@ -3768,7 +3769,7 @@
         <v>8.2100000000000006E-2</v>
       </c>
     </row>
-    <row r="259" spans="1:3">
+    <row r="259" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>4</v>
       </c>
@@ -3779,7 +3780,7 @@
         <v>4.58E-2</v>
       </c>
     </row>
-    <row r="260" spans="1:3">
+    <row r="260" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>4</v>
       </c>
@@ -3790,7 +3791,7 @@
         <v>8.3299999999999999E-2</v>
       </c>
     </row>
-    <row r="261" spans="1:3">
+    <row r="261" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>4</v>
       </c>
@@ -3801,7 +3802,7 @@
         <v>8.5599999999999996E-2</v>
       </c>
     </row>
-    <row r="262" spans="1:3">
+    <row r="262" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>4</v>
       </c>
@@ -3812,7 +3813,7 @@
         <v>4.7899999999999998E-2</v>
       </c>
     </row>
-    <row r="263" spans="1:3">
+    <row r="263" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>4</v>
       </c>
@@ -3823,7 +3824,7 @@
         <v>3.9600000000000003E-2</v>
       </c>
     </row>
-    <row r="264" spans="1:3">
+    <row r="264" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>4</v>
       </c>
@@ -3834,7 +3835,7 @@
         <v>7.7600000000000002E-2</v>
       </c>
     </row>
-    <row r="265" spans="1:3">
+    <row r="265" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>4</v>
       </c>
@@ -3845,7 +3846,7 @@
         <v>8.7900000000000006E-2</v>
       </c>
     </row>
-    <row r="266" spans="1:3">
+    <row r="266" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>4</v>
       </c>
@@ -3856,7 +3857,7 @@
         <v>6.6900000000000001E-2</v>
       </c>
     </row>
-    <row r="267" spans="1:3">
+    <row r="267" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>4</v>
       </c>
@@ -3867,7 +3868,7 @@
         <v>4.0500000000000001E-2</v>
       </c>
     </row>
-    <row r="268" spans="1:3">
+    <row r="268" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>4</v>
       </c>
@@ -3878,7 +3879,7 @@
         <v>0.1103</v>
       </c>
     </row>
-    <row r="269" spans="1:3">
+    <row r="269" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>4</v>
       </c>
@@ -3889,7 +3890,7 @@
         <v>4.6399999999999997E-2</v>
       </c>
     </row>
-    <row r="270" spans="1:3">
+    <row r="270" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>4</v>
       </c>
@@ -3900,7 +3901,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="271" spans="1:3">
+    <row r="271" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
         <v>4</v>
       </c>
@@ -3911,7 +3912,7 @@
         <v>3.5799999999999998E-2</v>
       </c>
     </row>
-    <row r="272" spans="1:3">
+    <row r="272" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
         <v>4</v>
       </c>
@@ -3922,7 +3923,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="273" spans="1:3">
+    <row r="273" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
         <v>4</v>
       </c>
@@ -3933,7 +3934,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="274" spans="1:3">
+    <row r="274" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
         <v>4</v>
       </c>
@@ -3944,7 +3945,7 @@
         <v>2.2700000000000001E-2</v>
       </c>
     </row>
-    <row r="275" spans="1:3">
+    <row r="275" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
         <v>4</v>
       </c>
@@ -3955,7 +3956,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="276" spans="1:3">
+    <row r="276" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
         <v>4</v>
       </c>
@@ -3966,7 +3967,7 @@
         <v>4.2900000000000001E-2</v>
       </c>
     </row>
-    <row r="277" spans="1:3">
+    <row r="277" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
         <v>4</v>
       </c>
@@ -3977,7 +3978,7 @@
         <v>6.9900000000000004E-2</v>
       </c>
     </row>
-    <row r="278" spans="1:3">
+    <row r="278" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
         <v>4</v>
       </c>
@@ -3988,7 +3989,7 @@
         <v>0.13</v>
       </c>
     </row>
-    <row r="279" spans="1:3">
+    <row r="279" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
         <v>4</v>
       </c>
@@ -3999,7 +4000,7 @@
         <v>5.6399999999999999E-2</v>
       </c>
     </row>
-    <row r="280" spans="1:3">
+    <row r="280" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
         <v>4</v>
       </c>
@@ -4010,7 +4011,7 @@
         <v>0.1077</v>
       </c>
     </row>
-    <row r="281" spans="1:3">
+    <row r="281" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
         <v>4</v>
       </c>
@@ -4021,7 +4022,7 @@
         <v>4.4400000000000002E-2</v>
       </c>
     </row>
-    <row r="282" spans="1:3">
+    <row r="282" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
         <v>4</v>
       </c>
@@ -4032,7 +4033,7 @@
         <v>9.74E-2</v>
       </c>
     </row>
-    <row r="283" spans="1:3">
+    <row r="283" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
         <v>4</v>
       </c>
@@ -4043,7 +4044,7 @@
         <v>3.2399999999999998E-2</v>
       </c>
     </row>
-    <row r="284" spans="1:3">
+    <row r="284" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
         <v>4</v>
       </c>
@@ -4054,7 +4055,7 @@
         <v>7.8700000000000006E-2</v>
       </c>
     </row>
-    <row r="285" spans="1:3">
+    <row r="285" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
         <v>4</v>
       </c>
@@ -4065,7 +4066,7 @@
         <v>7.5300000000000006E-2</v>
       </c>
     </row>
-    <row r="286" spans="1:3">
+    <row r="286" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
         <v>4</v>
       </c>
@@ -4076,7 +4077,7 @@
         <v>7.4499999999999997E-2</v>
       </c>
     </row>
-    <row r="287" spans="1:3">
+    <row r="287" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
         <v>4</v>
       </c>
@@ -4087,7 +4088,7 @@
         <v>2.9899999999999999E-2</v>
       </c>
     </row>
-    <row r="288" spans="1:3">
+    <row r="288" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
         <v>4</v>
       </c>
@@ -4098,7 +4099,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="289" spans="1:4">
+    <row r="289" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
         <v>4</v>
       </c>
@@ -4109,7 +4110,7 @@
         <v>7.4099999999999999E-2</v>
       </c>
     </row>
-    <row r="290" spans="1:4">
+    <row r="290" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
         <v>4</v>
       </c>
@@ -4120,7 +4121,7 @@
         <v>4.2299999999999997E-2</v>
       </c>
     </row>
-    <row r="291" spans="1:4">
+    <row r="291" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
         <v>4</v>
       </c>
@@ -4131,7 +4132,7 @@
         <v>8.2000000000000007E-3</v>
       </c>
     </row>
-    <row r="292" spans="1:4">
+    <row r="292" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
         <v>4</v>
       </c>
@@ -4142,7 +4143,7 @@
         <v>2.5700000000000001E-2</v>
       </c>
     </row>
-    <row r="293" spans="1:4">
+    <row r="293" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
         <v>4</v>
       </c>
@@ -4153,7 +4154,7 @@
         <v>1.55E-2</v>
       </c>
     </row>
-    <row r="294" spans="1:4">
+    <row r="294" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
         <v>4</v>
       </c>
@@ -4164,7 +4165,7 @@
         <v>3.4799999999999998E-2</v>
       </c>
     </row>
-    <row r="295" spans="1:4">
+    <row r="295" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
         <v>4</v>
       </c>
@@ -4175,7 +4176,7 @@
         <v>2.1499999999999998E-2</v>
       </c>
     </row>
-    <row r="296" spans="1:4">
+    <row r="296" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
         <v>4</v>
       </c>
@@ -4186,7 +4187,7 @@
         <v>2.01E-2</v>
       </c>
     </row>
-    <row r="297" spans="1:4">
+    <row r="297" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
         <v>4</v>
       </c>
@@ -4197,7 +4198,7 @@
         <v>3.1399999999999997E-2</v>
       </c>
     </row>
-    <row r="298" spans="1:4">
+    <row r="298" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
         <v>4</v>
       </c>
@@ -4211,7 +4212,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="299" spans="1:4">
+    <row r="299" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
         <v>4</v>
       </c>
@@ -4222,7 +4223,7 @@
         <v>2.3699999999999999E-2</v>
       </c>
     </row>
-    <row r="300" spans="1:4">
+    <row r="300" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
         <v>4</v>
       </c>
@@ -4233,7 +4234,7 @@
         <v>5.3400000000000003E-2</v>
       </c>
     </row>
-    <row r="301" spans="1:4">
+    <row r="301" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
         <v>4</v>
       </c>
@@ -4244,7 +4245,7 @@
         <v>1.06E-2</v>
       </c>
     </row>
-    <row r="302" spans="1:4">
+    <row r="302" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A302" t="s">
         <v>4</v>
       </c>
@@ -4255,7 +4256,7 @@
         <v>2.76E-2</v>
       </c>
     </row>
-    <row r="303" spans="1:4">
+    <row r="303" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A303" t="s">
         <v>4</v>
       </c>
@@ -4266,7 +4267,7 @@
         <v>2.64E-2</v>
       </c>
     </row>
-    <row r="304" spans="1:4">
+    <row r="304" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A304" t="s">
         <v>4</v>
       </c>
@@ -4277,7 +4278,7 @@
         <v>4.7999999999999996E-3</v>
       </c>
     </row>
-    <row r="305" spans="1:4">
+    <row r="305" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>4</v>
       </c>
@@ -4288,7 +4289,7 @@
         <v>2.8799999999999999E-2</v>
       </c>
     </row>
-    <row r="306" spans="1:4">
+    <row r="306" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>4</v>
       </c>
@@ -4299,7 +4300,7 @@
         <v>2.12E-2</v>
       </c>
     </row>
-    <row r="307" spans="1:4">
+    <row r="307" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>4</v>
       </c>
@@ -4310,7 +4311,7 @@
         <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="308" spans="1:4">
+    <row r="308" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>4</v>
       </c>
@@ -4321,7 +4322,7 @@
         <v>4.4499999999999998E-2</v>
       </c>
     </row>
-    <row r="309" spans="1:4">
+    <row r="309" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>4</v>
       </c>
@@ -4332,7 +4333,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="310" spans="1:4">
+    <row r="310" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>4</v>
       </c>
@@ -4343,7 +4344,7 @@
         <v>5.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="311" spans="1:4">
+    <row r="311" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>4</v>
       </c>
@@ -4354,7 +4355,7 @@
         <v>1.83E-2</v>
       </c>
     </row>
-    <row r="312" spans="1:4">
+    <row r="312" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>4</v>
       </c>
@@ -4365,7 +4366,7 @@
         <v>6.3E-3</v>
       </c>
     </row>
-    <row r="313" spans="1:4">
+    <row r="313" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>4</v>
       </c>
@@ -4376,7 +4377,7 @@
         <v>2.1700000000000001E-2</v>
       </c>
     </row>
-    <row r="314" spans="1:4">
+    <row r="314" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>4</v>
       </c>
@@ -4390,7 +4391,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="315" spans="1:4">
+    <row r="315" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>4</v>
       </c>
@@ -4401,7 +4402,7 @@
         <v>9.4999999999999998E-3</v>
       </c>
     </row>
-    <row r="316" spans="1:4">
+    <row r="316" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>4</v>
       </c>
@@ -4412,7 +4413,7 @@
         <v>3.4500000000000003E-2</v>
       </c>
     </row>
-    <row r="317" spans="1:4">
+    <row r="317" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>4</v>
       </c>
@@ -4423,7 +4424,7 @@
         <v>1.5699999999999999E-2</v>
       </c>
     </row>
-    <row r="318" spans="1:4">
+    <row r="318" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>4</v>
       </c>
@@ -4434,7 +4435,7 @@
         <v>3.6499999999999998E-2</v>
       </c>
     </row>
-    <row r="319" spans="1:4">
+    <row r="319" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>4</v>
       </c>
@@ -4445,7 +4446,7 @@
         <v>1.35E-2</v>
       </c>
     </row>
-    <row r="320" spans="1:4">
+    <row r="320" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>4</v>
       </c>
@@ -4456,7 +4457,7 @@
         <v>1.2200000000000001E-2</v>
       </c>
     </row>
-    <row r="321" spans="1:4">
+    <row r="321" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>4</v>
       </c>
@@ -4467,7 +4468,7 @@
         <v>1.7999999999999999E-2</v>
       </c>
     </row>
-    <row r="322" spans="1:4">
+    <row r="322" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>4</v>
       </c>
@@ -4478,7 +4479,7 @@
         <v>0.11940000000000001</v>
       </c>
     </row>
-    <row r="323" spans="1:4">
+    <row r="323" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>4</v>
       </c>
@@ -4489,7 +4490,7 @@
         <v>2.35E-2</v>
       </c>
     </row>
-    <row r="324" spans="1:4">
+    <row r="324" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>4</v>
       </c>
@@ -4500,7 +4501,7 @@
         <v>1.7600000000000001E-2</v>
       </c>
     </row>
-    <row r="325" spans="1:4">
+    <row r="325" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>4</v>
       </c>
@@ -4511,7 +4512,7 @@
         <v>9.4500000000000001E-2</v>
       </c>
     </row>
-    <row r="326" spans="1:4">
+    <row r="326" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>4</v>
       </c>
@@ -4522,7 +4523,7 @@
         <v>7.4399999999999994E-2</v>
       </c>
     </row>
-    <row r="327" spans="1:4">
+    <row r="327" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>4</v>
       </c>
@@ -4533,7 +4534,7 @@
         <v>6.3200000000000006E-2</v>
       </c>
     </row>
-    <row r="328" spans="1:4">
+    <row r="328" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>4</v>
       </c>
@@ -4547,7 +4548,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="329" spans="1:4">
+    <row r="329" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>4</v>
       </c>
@@ -4558,7 +4559,7 @@
         <v>0.11459999999999999</v>
       </c>
     </row>
-    <row r="330" spans="1:4">
+    <row r="330" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>4</v>
       </c>
@@ -4569,7 +4570,7 @@
         <v>0.18160000000000001</v>
       </c>
     </row>
-    <row r="331" spans="1:4">
+    <row r="331" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>4</v>
       </c>
@@ -4580,7 +4581,7 @@
         <v>2.75E-2</v>
       </c>
     </row>
-    <row r="332" spans="1:4">
+    <row r="332" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A332" t="s">
         <v>4</v>
       </c>
@@ -4591,7 +4592,7 @@
         <v>0.10199999999999999</v>
       </c>
     </row>
-    <row r="333" spans="1:4">
+    <row r="333" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
         <v>4</v>
       </c>
@@ -4602,7 +4603,7 @@
         <v>9.3200000000000005E-2</v>
       </c>
     </row>
-    <row r="334" spans="1:4">
+    <row r="334" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
         <v>4</v>
       </c>
@@ -4613,7 +4614,7 @@
         <v>6.2199999999999998E-2</v>
       </c>
     </row>
-    <row r="335" spans="1:4">
+    <row r="335" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
         <v>4</v>
       </c>
@@ -4624,7 +4625,7 @@
         <v>4.9000000000000002E-2</v>
       </c>
     </row>
-    <row r="336" spans="1:4">
+    <row r="336" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A336" t="s">
         <v>4</v>
       </c>
@@ -4635,7 +4636,7 @@
         <v>8.2199999999999995E-2</v>
       </c>
     </row>
-    <row r="337" spans="1:3">
+    <row r="337" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
         <v>4</v>
       </c>
@@ -4646,7 +4647,7 @@
         <v>8.1100000000000005E-2</v>
       </c>
     </row>
-    <row r="338" spans="1:3">
+    <row r="338" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
         <v>4</v>
       </c>
@@ -4657,7 +4658,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="339" spans="1:3">
+    <row r="339" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
         <v>4</v>
       </c>
@@ -4668,7 +4669,7 @@
         <v>5.6300000000000003E-2</v>
       </c>
     </row>
-    <row r="340" spans="1:3">
+    <row r="340" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
         <v>4</v>
       </c>
@@ -4679,7 +4680,7 @@
         <v>7.22E-2</v>
       </c>
     </row>
-    <row r="341" spans="1:3">
+    <row r="341" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
         <v>4</v>
       </c>
@@ -4690,7 +4691,7 @@
         <v>8.1100000000000005E-2</v>
       </c>
     </row>
-    <row r="342" spans="1:3">
+    <row r="342" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
         <v>4</v>
       </c>
@@ -4701,7 +4702,7 @@
         <v>6.13E-2</v>
       </c>
     </row>
-    <row r="343" spans="1:3">
+    <row r="343" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A343" t="s">
         <v>4</v>
       </c>
@@ -4712,7 +4713,7 @@
         <v>6.0699999999999997E-2</v>
       </c>
     </row>
-    <row r="344" spans="1:3">
+    <row r="344" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A344" t="s">
         <v>4</v>
       </c>
@@ -4723,7 +4724,7 @@
         <v>0.128</v>
       </c>
     </row>
-    <row r="345" spans="1:3">
+    <row r="345" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A345" t="s">
         <v>4</v>
       </c>
@@ -4734,7 +4735,7 @@
         <v>6.6400000000000001E-2</v>
       </c>
     </row>
-    <row r="346" spans="1:3">
+    <row r="346" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A346" t="s">
         <v>4</v>
       </c>
@@ -4745,7 +4746,7 @@
         <v>9.9299999999999999E-2</v>
       </c>
     </row>
-    <row r="347" spans="1:3">
+    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A347" t="s">
         <v>4</v>
       </c>
@@ -4756,7 +4757,7 @@
         <v>2.1100000000000001E-2</v>
       </c>
     </row>
-    <row r="348" spans="1:3">
+    <row r="348" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A348" t="s">
         <v>4</v>
       </c>
@@ -4767,7 +4768,7 @@
         <v>3.56E-2</v>
       </c>
     </row>
-    <row r="349" spans="1:3">
+    <row r="349" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A349" t="s">
         <v>4</v>
       </c>
@@ -4778,7 +4779,7 @@
         <v>0.10390000000000001</v>
       </c>
     </row>
-    <row r="350" spans="1:3">
+    <row r="350" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A350" t="s">
         <v>4</v>
       </c>
@@ -4789,7 +4790,7 @@
         <v>0.10050000000000001</v>
       </c>
     </row>
-    <row r="351" spans="1:3">
+    <row r="351" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A351" t="s">
         <v>4</v>
       </c>
@@ -4800,7 +4801,7 @@
         <v>5.4399999999999997E-2</v>
       </c>
     </row>
-    <row r="352" spans="1:3">
+    <row r="352" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A352" t="s">
         <v>4</v>
       </c>
@@ -4811,7 +4812,7 @@
         <v>0.14899999999999999</v>
       </c>
     </row>
-    <row r="353" spans="1:3">
+    <row r="353" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A353" t="s">
         <v>4</v>
       </c>
@@ -4822,7 +4823,7 @@
         <v>5.4100000000000002E-2</v>
       </c>
     </row>
-    <row r="354" spans="1:3">
+    <row r="354" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A354" t="s">
         <v>4</v>
       </c>
@@ -4833,7 +4834,7 @@
         <v>4.07E-2</v>
       </c>
     </row>
-    <row r="355" spans="1:3">
+    <row r="355" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A355" t="s">
         <v>4</v>
       </c>
@@ -4844,7 +4845,7 @@
         <v>1.0200000000000001E-2</v>
       </c>
     </row>
-    <row r="356" spans="1:3">
+    <row r="356" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A356" t="s">
         <v>4</v>
       </c>
@@ -4855,7 +4856,7 @@
         <v>7.2999999999999995E-2</v>
       </c>
     </row>
-    <row r="357" spans="1:3">
+    <row r="357" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A357" t="s">
         <v>4</v>
       </c>
@@ -4866,7 +4867,7 @@
         <v>3.0800000000000001E-2</v>
       </c>
     </row>
-    <row r="358" spans="1:3">
+    <row r="358" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A358" t="s">
         <v>4</v>
       </c>
@@ -4877,7 +4878,7 @@
         <v>3.7199999999999997E-2</v>
       </c>
     </row>
-    <row r="359" spans="1:3">
+    <row r="359" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A359" t="s">
         <v>4</v>
       </c>
@@ -4888,7 +4889,7 @@
         <v>2.8799999999999999E-2</v>
       </c>
     </row>
-    <row r="360" spans="1:3">
+    <row r="360" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A360" t="s">
         <v>4</v>
       </c>
@@ -4899,7 +4900,7 @@
         <v>3.2599999999999997E-2</v>
       </c>
     </row>
-    <row r="361" spans="1:3">
+    <row r="361" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A361" t="s">
         <v>4</v>
       </c>
@@ -4910,7 +4911,7 @@
         <v>3.1699999999999999E-2</v>
       </c>
     </row>
-    <row r="362" spans="1:3">
+    <row r="362" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A362" t="s">
         <v>4</v>
       </c>
@@ -4921,7 +4922,7 @@
         <v>3.1099999999999999E-2</v>
       </c>
     </row>
-    <row r="363" spans="1:3">
+    <row r="363" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A363" t="s">
         <v>4</v>
       </c>
@@ -4932,7 +4933,7 @@
         <v>1.17E-2</v>
       </c>
     </row>
-    <row r="364" spans="1:3">
+    <row r="364" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A364" t="s">
         <v>4</v>
       </c>
@@ -4943,7 +4944,7 @@
         <v>3.3399999999999999E-2</v>
       </c>
     </row>
-    <row r="365" spans="1:3">
+    <row r="365" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A365" t="s">
         <v>4</v>
       </c>
@@ -4954,7 +4955,7 @@
         <v>2.9899999999999999E-2</v>
       </c>
     </row>
-    <row r="366" spans="1:3">
+    <row r="366" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A366" t="s">
         <v>4</v>
       </c>
@@ -4965,7 +4966,7 @@
         <v>6.6000000000000003E-2</v>
       </c>
     </row>
-    <row r="367" spans="1:3">
+    <row r="367" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A367" t="s">
         <v>4</v>
       </c>
@@ -4976,7 +4977,7 @@
         <v>3.1300000000000001E-2</v>
       </c>
     </row>
-    <row r="368" spans="1:3">
+    <row r="368" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A368" t="s">
         <v>4</v>
       </c>
@@ -4987,7 +4988,7 @@
         <v>2.3599999999999999E-2</v>
       </c>
     </row>
-    <row r="369" spans="1:4">
+    <row r="369" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A369" t="s">
         <v>4</v>
       </c>
@@ -4998,7 +4999,7 @@
         <v>1.66E-2</v>
       </c>
     </row>
-    <row r="370" spans="1:4">
+    <row r="370" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A370" t="s">
         <v>4</v>
       </c>
@@ -5009,7 +5010,7 @@
         <v>2.9499999999999998E-2</v>
       </c>
     </row>
-    <row r="371" spans="1:4">
+    <row r="371" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A371" t="s">
         <v>4</v>
       </c>
@@ -5020,7 +5021,7 @@
         <v>1.1599999999999999E-2</v>
       </c>
     </row>
-    <row r="372" spans="1:4">
+    <row r="372" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A372" t="s">
         <v>4</v>
       </c>
@@ -5031,7 +5032,7 @@
         <v>4.4400000000000002E-2</v>
       </c>
     </row>
-    <row r="373" spans="1:4">
+    <row r="373" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A373" t="s">
         <v>4</v>
       </c>
@@ -5042,7 +5043,7 @@
         <v>2.0899999999999998E-2</v>
       </c>
     </row>
-    <row r="374" spans="1:4">
+    <row r="374" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A374" t="s">
         <v>4</v>
       </c>
@@ -5053,7 +5054,7 @@
         <v>6.4199999999999993E-2</v>
       </c>
     </row>
-    <row r="375" spans="1:4">
+    <row r="375" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A375" t="s">
         <v>4</v>
       </c>
@@ -5064,7 +5065,7 @@
         <v>2.5499999999999998E-2</v>
       </c>
     </row>
-    <row r="376" spans="1:4">
+    <row r="376" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A376" t="s">
         <v>4</v>
       </c>
@@ -5078,7 +5079,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="377" spans="1:4">
+    <row r="377" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A377" t="s">
         <v>4</v>
       </c>
@@ -5089,7 +5090,7 @@
         <v>2.98E-2</v>
       </c>
     </row>
-    <row r="378" spans="1:4">
+    <row r="378" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A378" t="s">
         <v>4</v>
       </c>
@@ -5100,7 +5101,7 @@
         <v>2.06E-2</v>
       </c>
     </row>
-    <row r="379" spans="1:4">
+    <row r="379" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A379" t="s">
         <v>4</v>
       </c>
@@ -5111,7 +5112,7 @@
         <v>1.8599999999999998E-2</v>
       </c>
     </row>
-    <row r="380" spans="1:4">
+    <row r="380" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A380" t="s">
         <v>4</v>
       </c>
@@ -5122,7 +5123,7 @@
         <v>4.6100000000000002E-2</v>
       </c>
     </row>
-    <row r="381" spans="1:4">
+    <row r="381" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A381" t="s">
         <v>4</v>
       </c>
@@ -5133,7 +5134,7 @@
         <v>1.83E-2</v>
       </c>
     </row>
-    <row r="382" spans="1:4">
+    <row r="382" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A382" t="s">
         <v>4</v>
       </c>
@@ -5144,7 +5145,7 @@
         <v>4.2599999999999999E-2</v>
       </c>
     </row>
-    <row r="383" spans="1:4">
+    <row r="383" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A383" t="s">
         <v>4</v>
       </c>
@@ -5155,7 +5156,7 @@
         <v>3.3099999999999997E-2</v>
       </c>
     </row>
-    <row r="384" spans="1:4">
+    <row r="384" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A384" t="s">
         <v>4</v>
       </c>
@@ -5166,7 +5167,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="385" spans="1:4">
+    <row r="385" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A385" t="s">
         <v>4</v>
       </c>
@@ -5177,7 +5178,7 @@
         <v>3.6900000000000002E-2</v>
       </c>
     </row>
-    <row r="386" spans="1:4">
+    <row r="386" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A386" t="s">
         <v>4</v>
       </c>
@@ -5191,7 +5192,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="387" spans="1:4">
+    <row r="387" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A387" t="s">
         <v>4</v>
       </c>
@@ -5205,7 +5206,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="388" spans="1:4">
+    <row r="388" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A388" t="s">
         <v>4</v>
       </c>
@@ -5216,7 +5217,7 @@
         <v>1.46E-2</v>
       </c>
     </row>
-    <row r="389" spans="1:4">
+    <row r="389" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A389" t="s">
         <v>4</v>
       </c>
@@ -5230,7 +5231,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="390" spans="1:4">
+    <row r="390" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A390" t="s">
         <v>4</v>
       </c>

</xml_diff>